<commit_message>
Align all workbook generators to the LLD spec theme
gen_template.py is the reference: title band 1F4E79 Calibri 12 bold
white, header row DDEBF7 dark bold Calibri 10, input cells FFFCE5,
borders B4B4B4, notes 595959 italic. envtree (ipam/checklist/config-book
headers) and gen_questionnaire adopted it; the questionnaire keeps its
category band D6E4F0 as the one section-level accent (same blue family).
Questionnaire regenerated; coverage check green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017F9N9oxYa81hgj1kB5MNFw
</commit_message>
<xml_diff>
--- a/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
+++ b/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,36 +32,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="001F4E79"/>
       <sz val="11"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="001F4E79"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00606060"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00909090"/>
+      <color rgb="00595959"/>
     </font>
   </fonts>
   <fills count="6">
@@ -73,12 +70,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -88,7 +85,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E3"/>
+        <fgColor rgb="00FFFCE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,23 +99,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00B4B4B4"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00B4B4B4"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00B4B4B4"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="00B4B4B4"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -144,10 +141,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -627,7 +621,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Version 1.0 - generated 2026-08-30 - schema 2.2</t>
+          <t>Version 1.0 - generated 2026-08-31 - schema 2.2</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1846,7 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>One row per workload per environment. Fill what you know; leave the rest blank.</t>
         </is>
@@ -1891,32 +1885,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>(example) Customer portal</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>prod</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>app-portal-prod</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Workloads/Prod</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>cloud-portal-prod@example.com</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Internet-facing</t>
         </is>
@@ -2115,7 +2109,7 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Known allocations and ranges to avoid. Scope: supernet offered to Huawei Cloud, an existing on-prem/other-cloud range to avoid, or a specific VPC you want pinned.</t>
         </is>
@@ -2149,27 +2143,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>(example) supernet</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>10.20.0.0/16</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Huawei Cloud allocation</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Nothing else uses this block</t>
         </is>
@@ -2349,7 +2343,7 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>One row per team. Access level: admin / power user / read-only / custom (describe in Notes).</t>
         </is>
@@ -2388,32 +2382,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>(example) Platform engineering</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Landing zone, network, shared services</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Alice Tan &lt;alice@example.com&gt;</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>all accounts</t>
         </is>
       </c>
-      <c r="F4" s="10" t="n"/>
+      <c r="F4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>

</xml_diff>

<commit_message>
Green section bands across the document family
The template's C6E0B4/375623 section device now appears wherever sections
exist: questionnaire category bands and config-book sections (shared
SEC_FONT/SEC_FILL in envtree). ipam/checklist have no section concept and
stay title+header only. Questionnaire regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017F9N9oxYa81hgj1kB5MNFw
</commit_message>
<xml_diff>
--- a/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
+++ b/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
@@ -53,8 +53,9 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E79"/>
+      <color rgb="00375623"/>
     </font>
     <font>
       <i val="1"/>
@@ -80,7 +81,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
     <fill>

</xml_diff>

<commit_message>
questionnaire: naming + enterprise-project questions, example-response column
- dedicated resource-naming question (was folded into the email question);
  the draft build infers every resource name from the stated pattern
- new enterprise-project question (resource-group analogue) wired to
  CostCenters + AppPermissionSets; EP layout and tag plan inferred as
  single reviewable DEFAULTED items (questionnaire-to-spec skill rules)
- survey sheets gain an Example Response column (italic, falls back to
  default_if_silent); intake now locates Customer Response by header so
  forms filled on older templates still parse

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017F9N9oxYa81hgj1kB5MNFw
</commit_message>
<xml_diff>
--- a/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
+++ b/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00375623"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
     </font>
     <font>
       <i val="1"/>
@@ -116,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -139,10 +144,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -622,7 +630,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Version 1.0 - generated 2026-08-31 - schema 2.2</t>
+          <t>Version 1.0 - generated 2026-09-01 - schema 2.2</t>
         </is>
       </c>
     </row>
@@ -640,13 +648,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -669,10 +678,15 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Guidance &amp; Examples</t>
+          <t>Guidance</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Example Response</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Customer Response</t>
         </is>
@@ -685,7 +699,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="62" customHeight="1">
+    <row r="4" ht="76" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>C1</t>
@@ -701,9 +715,14 @@
           <t>Free text; attach an account inventory or org chart if you have one. This shapes the account and OU structure we propose.</t>
         </is>
       </c>
-      <c r="D4" s="8" t="n"/>
-    </row>
-    <row r="5" ht="62" customHeight="1">
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>AWS: ~25 accounts, one per team; Azure: 8 subscriptions (legacy ERP); no Huawei footprint yet.</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="n"/>
+    </row>
+    <row r="5" ht="76" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>C2</t>
@@ -719,7 +738,12 @@
           <t>Greenfield accounts give the cleanest governance baseline. If some accounts must be adopted as-is, list them and what they host.</t>
         </is>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Greenfield: a new organization with fresh core + workload accounts.</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="n"/>
     </row>
     <row r="6" ht="76" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -737,9 +761,14 @@
           <t>Appendix A (Accounts &amp; Environments) has a table for this if you prefer rows over prose. Per-environment accounts are our recommended isolation boundary.</t>
         </is>
       </c>
-      <c r="D6" s="8" t="n"/>
-    </row>
-    <row r="7" ht="62" customHeight="1">
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>One account per workload per environment tier.</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="76" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>C4</t>
@@ -755,9 +784,14 @@
           <t>A diagram or export is ideal. We mirror proven structure where it fits Huawei Organizations.</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="62" customHeight="1">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>AWS Control Tower: Security / Infrastructure / Workloads OUs. Worked well; too many SCP exceptions crept in.</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="76" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>C5</t>
@@ -773,7 +807,12 @@
           <t>e.g. ap-southeast-3 (Singapore) primary. Residency constraints become an org-wide region guardrail.</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Single region ap-southeast-3, region-lock guardrail staged (not enforced).</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n"/>
     </row>
     <row r="9" ht="76" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -783,191 +822,241 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>What naming and email conventions should we follow? Each Huawei account needs a globally unique email address - do you have a pattern (e.g. cloud-&lt;account&gt;@yourco.com), and do you have a resource-naming standard?</t>
+          <t>What email convention should account mailboxes follow? Each Huawei account needs a globally unique email address - do you have a pattern (e.g. cloud-&lt;account&gt;@yourco.com)?</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Plus-addressing (team+lz-prod@yourco.com) works if your mail system supports it. If you have no standard, we apply Huawei best-practice naming.</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+          <t>Plus-addressing (team+lz-prod@yourco.com) works if your mail system supports it.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>cloud-&lt;account&gt;@acme.com, e.g. cloud-lz-prod@acme.com (plus-addressing not supported).</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="104" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Do you have a cloud resource naming convention (VPCs, subnets, gateways, buckets, vaults, log groups, ...)? State the pattern and an example, e.g. &lt;org&gt;-&lt;region&gt;-&lt;env&gt;-&lt;service&gt;-&lt;nn&gt; -&gt; acme-sg-prd-vpc-01.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Every named resource in the draft design is generated from this pattern, so one answer names the whole estate consistently. Note any hard limits (bucket names are globally unique and lowercase; some services cap length).</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>&lt;org&gt;-&lt;region&gt;-&lt;env&gt;-&lt;service&gt;-&lt;nn&gt;, e.g. acme-sg-prd-vpc-01; buckets lowercase with acme- prefix.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Identity &amp; Access</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>C7</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Which teams will work in the cloud (platform, application, security, network, database, finance, ...) and what is each team responsible for?</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Appendix C (Teams &amp; Access) has a table for this. Teams map to Identity Center groups and permission sets.</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="76" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>C8</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Platform team (LZ + network), AppDev (portal), SecOps (SOC + audit), DBA; finance needs read-only cost views.</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>How should people sign in to Huawei Cloud: federated through your corporate identity provider (Entra ID / AD FS / Okta / other), or as natively managed Identity Center users? Which IdP product and version do you run?</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Federation keeps joiner-mover-leaver in your IdP. Native IC users need no IdP integration but are managed separately.</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Native Identity Center users until IdP federation is confirmed.</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Does your identity provider support SAML 2.0 for sign-in and SCIM for automatic user/group provisioning?</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Both supported: full federation with auto-provisioning. SAML only: federation with manual user sync.</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="62" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>C10</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Entra ID - SAML 2.0 and SCIM both available.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="76" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Do third parties (vendors, MSPs, auditors, outsourced developers) need access? Who, to which accounts or applications, at what permission level, and standing or time-boxed?</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Third-party access gets its own groups and least-privilege permission sets so it can be revoked cleanly.</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="62" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>C11</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>No third-party access provisioned.</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n"/>
+    </row>
+    <row r="16" ht="76" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>What password, MFA and session policies must the cloud enforce? (minimum length, expiry, MFA mandatory for whom, console session timeout, lockout rules)</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>If you have no written policy, we apply the LZ baseline: 12+ character passwords, 90-day expiry, MFA required, 8-hour sessions, 60-minute console timeout.</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>LZ baseline hardening policy.</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Network</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="62" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>C12</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+    <row r="18" ht="62" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Describe your current network: data centres, offices, existing cloud networks, and how they interconnect. Attach a topology diagram if one exists.</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Even a rough sketch helps. This anchors the hub-and-spoke design and interconnect plan.</t>
         </is>
       </c>
-      <c r="D17" s="8" t="n"/>
-    </row>
-    <row r="18" ht="76" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>C13</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Two DCs (SG + KL) linked by MPLS; AWS VPCs reach on-prem via Transit Gateway; offices on SD-WAN.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="76" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Which connectivity do you need between Huawei Cloud and your on-premises sites or other clouds? Private line (Direct Connect), site-to-site VPN, or both - and does the link need high availability?</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>List each site/cloud that must reach Huawei Cloud. VPN specifics (devices, IPs, routing) come in the deep-dive section.</t>
         </is>
       </c>
-      <c r="D18" s="8" t="n"/>
-    </row>
-    <row r="19" ht="62" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>No hybrid connectivity provisioned.</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="76" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>How should internet access work? Which applications need outbound internet, which must be reachable from the internet, and is centralized egress through a hub NAT + firewall acceptable?</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Centralized egress is the LZ default: all spoke traffic exits through the inspected hub. Exceptions need a stated reason.</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n"/>
-    </row>
-    <row r="20" ht="62" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>The design connects VPCs hub-and-spoke through an Enterprise Router, which charges per attachment and per GB of traffic. Any objection, or constraints on inter-VPC bandwidth or cost?</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>The alternative (VPC peering mesh) does not scale with accounts and bypasses central inspection.</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="n"/>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Centralized egress via hub NAT behind the cloud firewall.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n"/>
     </row>
     <row r="21" ht="76" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -977,33 +1066,43 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
+          <t>The design connects VPCs hub-and-spoke through an Enterprise Router, which charges per attachment and per GB of traffic. Any objection, or constraints on inter-VPC bandwidth or cost?</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>The alternative (VPC peering mesh) does not scale with accounts and bypasses central inspection.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Enterprise Router hub-and-spoke accepted.</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
           <t>IP addressing: can you allocate Huawei Cloud a dedicated private supernet (e.g. a /16 or larger) that overlaps nothing on-premises or in other clouds? Should your team or Huawei plan the per-VPC subnets within it?</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Appendix B (IP Plan) has a table for known allocations and ranges to avoid. We recommend one supernet, centrally carved.</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="62" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>C17</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>How many VPCs do you expect per account - one per account, one per environment, or several per application? Any reason to deviate from one VPC per workload account?</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>One VPC per workload account is the LZ default; the account boundary already isolates environments.</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="n"/>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>10.20.0.0/16 reserved for Huawei Cloud (on-prem uses 10.0-10.19); Huawei plans the subnets.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n"/>
     </row>
     <row r="23" ht="62" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -1013,94 +1112,119 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
+          <t>How many VPCs do you expect per account - one per account, one per environment, or several per application? Any reason to deviate from one VPC per workload account?</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>One VPC per workload account is the LZ default; the account boundary already isolates environments.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>One VPC per workload account.</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="76" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
           <t>Which applications must communicate with each other, and which must be isolated? If you have a communication matrix (source, destination, port, protocol), attach it.</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>This drives firewall policy and security-group rules. No matrix: state the rule of thumb, e.g. 'prod isolated from non-prod; shared services reachable by all'.</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n"/>
-    </row>
-    <row r="24" ht="62" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>C19</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Default-deny between applications; shared services reachable by all.</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="76" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Which tags must every cloud resource carry (e.g. project, owner, environment, cost-centre), and should resource creation be blocked when mandatory tags are missing?</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Tag keys/values feed cost allocation and the tag-enforcement guardrail. Blocking untagged creation is strict but keeps the estate clean from day one.</t>
         </is>
       </c>
-      <c r="D24" s="8" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>project/owner/env/bu tagged by the platform; enforcement staged, not blocking.</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="62" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>C20</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Which security products do you use today (perimeter firewalls, EDR, SIEM, vulnerability management, PAM), and which must carry over or integrate with the cloud?</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>e.g. an existing PAM/bastion that must reach cloud servers, or an IPS policy to replicate.</t>
         </is>
       </c>
-      <c r="D26" s="8" t="n"/>
-    </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>C21</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Palo Alto perimeter, CrowdStrike EDR, Splunk SIEM - EDR and SIEM must extend to cloud servers.</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="104" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Cloud Firewall expectations: should intrusion prevention observe first or block immediately? Do you want antivirus scanning at the perimeter? Should the firewall notify on attack detections and high traffic - and to whom? Billing: pay-per-use or monthly subscription?</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>Default rollout: IPS in observe mode first, then block after tuning; attack + high-traffic alerts to the ops mailbox; pay-per-use until sizing is proven.</t>
         </is>
       </c>
-      <c r="D27" s="8" t="n"/>
-    </row>
-    <row r="28" ht="76" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>C22</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Do you need a cloud security-operations workspace (SecMaster) for centralized alerts and incident handling? Host security (HSS) on servers? Database security (DBSS)? Who consumes the alerts day-to-day?</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>SecMaster carries a monthly cost per workspace; HSS/DBSS are per-instance quotas.</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="n"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>IPS observe mode, alarms on to the ops topic, pay-per-use.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n"/>
     </row>
     <row r="29" ht="76" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -1110,40 +1234,50 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
+          <t>Do you need a cloud security-operations workspace (SecMaster) for centralized alerts and incident handling? Host security (HSS) on servers? Database security (DBSS)? Who consumes the alerts day-to-day?</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>SecMaster carries a monthly cost per workspace; HSS/DBSS are per-instance quotas.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>SecMaster in the security account; HSS/DBSS deferred.</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
           <t>Which actions should be hard-blocked organization-wide, for everyone including admins? Examples: leaving the organization, disabling audit logging, making storage public, creating resources outside approved regions.</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>These become service control policies (guardrails). We stage them in dry-run first, then enforce.</t>
         </is>
       </c>
-      <c r="D29" s="8" t="n"/>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>The 8 LZ baseline guardrails, staged (created, not enforced).</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Compliance &amp; Audit</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>C24</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Must every action in every account be logged centrally, tamper-proof and searchable? How long must audit logs be retained (hot and archived)?</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Common answer: 1 year online + long-term archive. Drives the central audit trail, its bucket and retention tiers.</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="n"/>
     </row>
     <row r="32" ht="62" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -1153,15 +1287,20 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Which regulatory or industry frameworks apply to you (e.g. MAS TRM, PDPA, PCI-DSS, ISO 27001, SOC 2), and do auditors need evidence reports from the cloud platform?</t>
+          <t>Must every action in every account be logged centrally, tamper-proof and searchable? How long must audit logs be retained (hot and archived)?</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Frameworks map to continuous-compliance rule packs evaluated against all accounts.</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="n"/>
+          <t>Common answer: 1 year online + long-term archive. Drives the central audit trail, its bucket and retention tiers.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Org-wide audit trail to the security account, 365-day retention.</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="n"/>
     </row>
     <row r="33" ht="62" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
@@ -1171,58 +1310,73 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
+          <t>Which regulatory or industry frameworks apply to you (e.g. MAS TRM, PDPA, PCI-DSS, ISO 27001, SOC 2), and do auditors need evidence reports from the cloud platform?</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Frameworks map to continuous-compliance rule packs evaluated against all accounts.</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>ISO 27001 + PDPA; auditors want a yearly conformance evidence export.</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="62" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
           <t>Do you run continuous compliance monitoring today (AWS Config rules, Azure Policy)? Which account/team should own compliance tooling and its findings on Huawei Cloud?</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Typically the security account owns the recorder, aggregator and rule packs.</t>
         </is>
       </c>
-      <c r="D33" s="8" t="n"/>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Config recorder + org aggregator in the security account.</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Operations &amp; Monitoring</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="62" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>C27</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
+    <row r="36" ht="76" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>How do you monitor infrastructure today: which metrics and logs are collected, with which tools (Zabbix, Prometheus, vendor consoles), and what alarm rules and on-call flow exist?</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>We map existing practice onto Cloud Eye one-click monitoring bundles + an alerting topic.</t>
         </is>
       </c>
-      <c r="D35" s="8" t="n"/>
-    </row>
-    <row r="36" ht="62" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>C28</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Should logs and monitoring from all accounts aggregate into one central operations account? Which log types matter most (audit, firewall, DNS, flow, application)?</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Central aggregation is the LZ default: member-account logs converge to the ops account and archive to object storage.</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="n"/>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Cloud Eye baseline bundles on core services, alerts to one ops topic.</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="n"/>
     </row>
     <row r="37" ht="62" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
@@ -1232,69 +1386,130 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
+          <t>Should logs and monitoring from all accounts aggregate into one central operations account? Which log types matter most (audit, firewall, DNS, flow, application)?</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Central aggregation is the LZ default: member-account logs converge to the ops account and archive to object storage.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>All platform logs converge centrally and archive to OBS.</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="62" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
           <t>Log retention: how long must each class of log stay hot/searchable, and how long in cheap archive storage? Any class that must move to deep archive after a period?</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>e.g. searchable 90 days, archived 1 year, deep-archived beyond. Drives retention tiers per log class.</t>
         </is>
       </c>
-      <c r="D37" s="8" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>90-day hot, 365-day archive.</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Finance &amp; Cost Management</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="48" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>C30</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
+    <row r="40" ht="62" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>C31</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Who manages cloud spend? Is there a financial administrator, and are budgets issued and controlled from the management account?</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>Shapes billing-account setup and who gets cost visibility.</t>
         </is>
       </c>
-      <c r="D39" s="8" t="n"/>
-    </row>
-    <row r="40" ht="48" customHeight="1">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>C31</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Central billing from the management account.</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n"/>
+    </row>
+    <row r="41" ht="62" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>C32</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Must cloud costs be allocated within your organization? Along which dimensions - business unit, department, project, environment, owner?</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Dimensions become cost-centre enterprise projects + the tag plan from the Network section.</t>
         </is>
       </c>
-      <c r="D40" s="8" t="n"/>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Cost centres per business unit, prod/dev typed.</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="n"/>
+    </row>
+    <row r="42" ht="104" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>C33</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>How should resources be grouped INSIDE accounts using Enterprise Projects - Huawei's in-account grouping construct (closest analogue: Azure resource groups, or AWS tag-based resource groups)? By application, environment, department, cost centre - or do you have no preference?</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise projects scope both cost reporting and permissions (an admin can be limited to one EP), so the grouping outlives billing. No preference: the design derives an EP layout from your workload and cost-allocation answers.</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Group by app + environment, e.g. portal-prd-ep / portal-uat-ep - mirrors our Azure resource-group layout.</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1306,13 +1521,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1335,10 +1551,15 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Guidance &amp; Examples</t>
+          <t>Guidance</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Example Response</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Customer Response</t>
         </is>
@@ -1368,6 +1589,7 @@
         </is>
       </c>
       <c r="D4" s="8" t="n"/>
+      <c r="E4" s="9" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1376,7 +1598,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="76" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>D2</t>
@@ -1392,9 +1614,14 @@
           <t>We strongly prefer OIDC/assume-role federation for pipelines; long-lived AK/SK is a last resort with rotation requirements.</t>
         </is>
       </c>
-      <c r="D6" s="8" t="n"/>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>GitHub Actions (cloud-hosted); OIDC federation preferred, no static keys in pipelines.</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="62" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>D3</t>
@@ -1410,9 +1637,14 @@
           <t>Informs custody of the management-account root user and the break-glass runbook.</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="76" customHeight="1">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Root credentials sealed with IT security, MFA on; every use requires a ticket and is reviewed.</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>D4</t>
@@ -1428,7 +1660,12 @@
           <t>App-scoped permission sets use enterprise-project scoping - more setup, tighter blast radius. Also note preferred session duration and a portal alias (the sign-in URL name) if you have one.</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Three standard tiers per account; no app-scoped sets.</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -1437,7 +1674,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="76" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>D5</t>
@@ -1453,9 +1690,14 @@
           <t>One answer block per site is fine. BGP with dual tunnels is our recommended HA pattern.</t>
         </is>
       </c>
-      <c r="D10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>HQ: Fortinet 200F, static IP, BGP (AS 65010), reach 10.0.0.0/12, ~200 Mbit/s, dual tunnels.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="62" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>D6</t>
@@ -1471,7 +1713,12 @@
           <t>Skip if single-region.</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n"/>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Skip - single region for now; DR ambition revisited next year.</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1489,9 +1736,14 @@
           <t>Default: an app subnet and a db subnet per VPC, plus small platform subnets the design adds automatically.</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="62" customHeight="1">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>app + db subnets per spoke VPC.</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="76" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>D8</t>
@@ -1507,9 +1759,14 @@
           <t>Skip if no containers planned.</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>CCE planned for the portal re-platform next year; reserve a /20 per cluster in the IP plan.</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="104" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>D9</t>
@@ -1525,7 +1782,12 @@
           <t>e.g. 'corp.internal on two on-prem DCs; cloud must resolve it; keep public zones at our registrar'. This shapes private zones, resolver endpoints and forwarding rules. Note whether DNS queries should be logged for security analytics.</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n"/>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Private zone + hybrid resolver; public DNS stays at the current registrar.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n"/>
     </row>
     <row r="15" ht="62" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -1543,7 +1805,12 @@
           <t>Each published app becomes a load-balancer/DNAT entry behind the firewall, optionally fronted by WAF.</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n"/>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>No inbound publishing provisioned.</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n"/>
     </row>
     <row r="16" ht="62" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -1561,9 +1828,14 @@
           <t>Sizes the egress/ingress EIPs. Default: one 100 Mbit/s bandwidth-billed egress EIP, grown on demand.</t>
         </is>
       </c>
-      <c r="D16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="48" customHeight="1">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1x 100 Mbit/s egress EIP, bandwidth-billed.</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="62" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>D12</t>
@@ -1579,7 +1851,12 @@
           <t>Flow logs add LTS log volume/cost. Default: enabled, 90-day hot retention.</t>
         </is>
       </c>
-      <c r="D17" s="8" t="n"/>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Flow logs on, 90-day retention.</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -1604,9 +1881,14 @@
           <t>Skip if no internet-facing web apps. A dedicated WAF instance lives in the hub DMZ in front of the ingress load balancer.</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n"/>
-    </row>
-    <row r="20" ht="48" customHeight="1">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>WAF off until an internet-facing app needs it.</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="62" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>D14</t>
@@ -1622,9 +1904,14 @@
           <t>Basic Anti-DDoS is free per public IP; we tune thresholds and alarms per EIP.</t>
         </is>
       </c>
-      <c r="D20" s="8" t="n"/>
-    </row>
-    <row r="21" ht="48" customHeight="1">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Default Anti-DDoS thresholds, no per-EIP tuning.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="62" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>D15</t>
@@ -1640,9 +1927,14 @@
           <t>Attach the lists or name the feed. These seed firewall blacklists/whitelists and domain groups.</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="48" customHeight="1">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>No seed lists; firewall starts with the rule baseline only.</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="62" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>D16</t>
@@ -1658,9 +1950,14 @@
           <t>The LZ encrypts audit/log storage with dedicated KMS keys by default; BYOK changes key custody.</t>
         </is>
       </c>
-      <c r="D22" s="8" t="n"/>
-    </row>
-    <row r="23" ht="48" customHeight="1">
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Platform-managed KMS keys per sensitive bucket.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="62" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>D17</t>
@@ -1676,7 +1973,12 @@
           <t>Default guardrail denies public storage outright; a tag-based exception path can be added with an approval process.</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Public storage denied outright, no exception path.</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -1701,7 +2003,12 @@
           <t>Exemptions reduce noise but create blind spots; name them explicitly.</t>
         </is>
       </c>
-      <c r="D25" s="8" t="n"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>No exemptions.</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -1710,7 +2017,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="62" customHeight="1">
+    <row r="27" ht="76" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>D19</t>
@@ -1726,7 +2033,12 @@
           <t>These become subscriptions on the central alerting topic (also used by firewall and DDoS alarms).</t>
         </is>
       </c>
-      <c r="D27" s="8" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>ops-team@acme.com (all severities); oncall SMS +65 9xxx xxxx (critical only).</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n"/>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -1744,7 +2056,12 @@
           <t>Cloud logs can be pulled from the central archive or streamed; the method affects the aggregation design.</t>
         </is>
       </c>
-      <c r="D28" s="8" t="n"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>No SIEM integration.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n"/>
     </row>
     <row r="29" ht="76" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -1762,7 +2079,12 @@
           <t>The LZ provisions the platform; workload backup policy is designed against these answers and lands with the workload rollout.</t>
         </is>
       </c>
-      <c r="D29" s="8" t="n"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>All servers nightly (RPO 24h); databases RPO 15 min; keep 30 days hot + 1 year archive.</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
@@ -1771,7 +2093,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="62" customHeight="1">
+    <row r="31" ht="76" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
           <t>D22</t>
@@ -1787,9 +2109,14 @@
           <t>Common pattern: platform costs absorbed centrally or split pro-rata by consumption.</t>
         </is>
       </c>
-      <c r="D31" s="8" t="n"/>
-    </row>
-    <row r="32" ht="62" customHeight="1">
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Platform costs absorbed centrally.</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="76" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
           <t>D23</t>
@@ -1805,18 +2132,23 @@
           <t>Commercial structure can constrain how accounts attach to billing; budget alerts reuse the ops alerting topic.</t>
         </is>
       </c>
-      <c r="D32" s="8" t="n"/>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Partner/reseller agreement via &lt;partner&gt;; alert finance@acme.com at 80% of monthly budget.</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A30:E30"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1886,32 +2218,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>(example) Customer portal</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>prod</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>app-portal-prod</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Workloads/Prod</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>cloud-portal-prod@example.com</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Internet-facing</t>
         </is>
@@ -2144,27 +2476,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>(example) supernet</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>10.20.0.0/16</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Huawei Cloud allocation</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Nothing else uses this block</t>
         </is>
@@ -2383,32 +2715,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>(example) Platform engineering</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Landing zone, network, shared services</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Alice Tan &lt;alice@example.com&gt;</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>all accounts</t>
         </is>
       </c>
-      <c r="F4" s="9" t="n"/>
+      <c r="F4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -2585,7 +2917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2765,19 +3097,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Huawei best-practice naming convention.</t>
+          <t>cloud-&lt;account&gt;@&lt;your-domain&gt; pattern proposed in the draft.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2787,30 +3119,34 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>01_Foundation.OrganizationalUnits; 01_Foundation.WorkloadAccounts</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>05_Network.HubVPCs.VPCName; 05_Network.HubSubnets.Name; 05_Network.SpokeVPCs.VPCName; 05_Network.EIPs.Name; 05_Network.NATGateways.Name; 06_Observability.AuditSettings; 08_DNS.ResolverEndpoints.Name</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Huawei best-practice naming (&lt;org&gt;-&lt;region&gt;-&lt;env&gt;-&lt;service&gt;-&lt;nn&gt;); all resource names inferred from it in the draft spec, flagged for review.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Identity &amp; Access</t>
+          <t>Organization &amp; Accounts</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>03_Identity.Groups</t>
+          <t>01_Foundation.OrganizationalUnits; 01_Foundation.WorkloadAccounts</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -2833,14 +3169,10 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>03_Identity.Settings; 03_Identity.Users</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Native Identity Center users until IdP federation is confirmed.</t>
-        </is>
-      </c>
+          <t>03_Identity.Groups</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2860,10 +3192,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>03_Identity.Settings</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>03_Identity.Settings; 03_Identity.Users</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Native Identity Center users until IdP federation is confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2883,14 +3219,10 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>03_Identity.PermissionSets; 03_Identity.AccountAssignments</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No third-party access provisioned.</t>
-        </is>
-      </c>
+          <t>03_Identity.Settings</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2910,24 +3242,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>03_Identity.Settings.ic_min_password_length; 03_Identity.Settings.ic_mfa_required</t>
+          <t>03_Identity.PermissionSets; 03_Identity.AccountAssignments</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LZ baseline hardening policy.</t>
+          <t>No third-party access provisioned.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2937,15 +3269,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>03_Identity.PermissionSets; 03_Identity.AppPermissionSets</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>03_Identity.Settings.ic_min_password_length; 03_Identity.Settings.ic_mfa_required</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LZ baseline hardening policy.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2960,7 +3296,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>03_Identity.Settings</t>
+          <t>03_Identity.PermissionSets; 03_Identity.AppPermissionSets</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -2968,7 +3304,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2983,37 +3319,37 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>03_Identity.PermissionSets; 03_Identity.AppPermissionSets; 03_Identity.AccountAssignments; 03_Identity.Settings.identity_center_alias</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Three standard tiers per account; no app-scoped sets.</t>
-        </is>
-      </c>
+          <t>03_Identity.Settings</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Network</t>
+          <t>Identity &amp; Access</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05_Network.HubVPCs</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>03_Identity.PermissionSets; 03_Identity.AppPermissionSets; 03_Identity.AccountAssignments; 03_Identity.Settings.identity_center_alias</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Three standard tiers per account; no app-scoped sets.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3033,14 +3369,10 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10_VPN.Gateways; 10_VPN.Connections; 10_VPN.Settings</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>No hybrid connectivity provisioned.</t>
-        </is>
-      </c>
+          <t>05_Network.HubVPCs</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3060,12 +3392,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05_Network.NATGateways; 05_Network.SNATRules; 05_Network.Settings.snat_vpc_attachment</t>
+          <t>10_VPN.Gateways; 10_VPN.Connections; 10_VPN.Settings</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Centralized egress via hub NAT behind the cloud firewall.</t>
+          <t>No hybrid connectivity provisioned.</t>
         </is>
       </c>
     </row>
@@ -3087,12 +3419,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05_Network.EnterpriseRouter; 05_Network.Settings</t>
+          <t>05_Network.NATGateways; 05_Network.SNATRules; 05_Network.Settings.snat_vpc_attachment</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Enterprise Router hub-and-spoke accepted.</t>
+          <t>Centralized egress via hub NAT behind the cloud firewall.</t>
         </is>
       </c>
     </row>
@@ -3114,12 +3446,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05_Network.Settings.spoke_private_supernet; 05_Network.HubVPCs; 05_Network.HubSubnets; 05_Network.SpokeVPCs; 05_Network.SpokeSubnets</t>
+          <t>05_Network.EnterpriseRouter; 05_Network.Settings</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Huawei plans subnets within a customer-provided supernet.</t>
+          <t>Enterprise Router hub-and-spoke accepted.</t>
         </is>
       </c>
     </row>
@@ -3141,12 +3473,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05_Network.SpokeVPCs</t>
+          <t>05_Network.Settings.spoke_private_supernet; 05_Network.HubVPCs; 05_Network.HubSubnets; 05_Network.SpokeVPCs; 05_Network.SpokeSubnets</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>One VPC per workload account.</t>
+          <t>Huawei plans subnets within a customer-provided supernet.</t>
         </is>
       </c>
     </row>
@@ -3168,12 +3500,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>09_CFW.ACLRules; 09_CFW.AddressGroups; 09_CFW.ServiceGroups; 11_SGACL.SecurityGroups; 11_SGACL.SGRules</t>
+          <t>05_Network.SpokeVPCs</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Default-deny between applications; shared services reachable by all.</t>
+          <t>One VPC per workload account.</t>
         </is>
       </c>
     </row>
@@ -3195,24 +3527,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Global.MasterDefaultTags; 01_Foundation.TagPolicies; 04_Perimeter.PredefinedTags; 04_Perimeter.SCPs.MandatoryTags; 01_Foundation.Settings.enforce_tag_keys_scp</t>
+          <t>09_CFW.ACLRules; 09_CFW.AddressGroups; 09_CFW.ServiceGroups; 11_SGACL.SecurityGroups; 11_SGACL.SGRules</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>project/owner/env/bu tagged by the platform; enforcement staged, not blocking.</t>
+          <t>Default-deny between applications; shared services reachable by all.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3222,15 +3554,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10_VPN.Gateways; 10_VPN.CustomerGateways; 10_VPN.Connections; 05_Network.EnterpriseRouter.er_asn</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>Global.MasterDefaultTags; 01_Foundation.TagPolicies; 04_Perimeter.PredefinedTags; 04_Perimeter.SCPs.MandatoryTags; 01_Foundation.Settings.enforce_tag_keys_scp</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>project/owner/env/bu tagged by the platform; enforcement staged, not blocking.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3243,13 +3579,17 @@
           <t>Network</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>10_VPN.Gateways; 10_VPN.CustomerGateways; 10_VPN.Connections; 05_Network.EnterpriseRouter.er_asn</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3262,21 +3602,13 @@
           <t>Network</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>05_Network.SpokeSubnets; 05_Network.HubSubnets</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>app + db subnets per spoke VPC.</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3291,15 +3623,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05_Network.SpokeVPCs</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>05_Network.SpokeSubnets; 05_Network.HubSubnets</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>app + db subnets per spoke VPC.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3314,19 +3650,15 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08_DNS.Settings; 08_DNS.PublicZones; 08_DNS.PrivateZones; 08_DNS.RecordSets; 08_DNS.ResolverEndpoints; 08_DNS.ResolverRules; 08_DNS.AccessLogs; 05_Network.Settings.subnet_dns_servers</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Private zone + hybrid resolver; public DNS stays at the current registrar.</t>
-        </is>
-      </c>
+          <t>05_Network.SpokeVPCs</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3341,19 +3673,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05_Network.DNATRules; 05_Network.ELBs</t>
+          <t>08_DNS.Settings; 08_DNS.PublicZones; 08_DNS.PrivateZones; 08_DNS.RecordSets; 08_DNS.ResolverEndpoints; 08_DNS.ResolverRules; 08_DNS.AccessLogs; 05_Network.Settings.subnet_dns_servers</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>No inbound publishing provisioned.</t>
+          <t>Private zone + hybrid resolver; public DNS stays at the current registrar.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3368,19 +3700,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05_Network.EIPs</t>
+          <t>05_Network.DNATRules; 05_Network.ELBs</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1x 100 Mbit/s egress EIP, bandwidth-billed.</t>
+          <t>No inbound publishing provisioned.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3395,37 +3727,41 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05_Network.Settings.enable_vpc_flow_logs; 05_Network.Settings.flow_log_retention_days</t>
+          <t>05_Network.EIPs</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Flow logs on, 90-day retention.</t>
+          <t>1x 100 Mbit/s egress EIP, bandwidth-billed.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>09_CFW.Settings</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>05_Network.Settings.enable_vpc_flow_logs; 05_Network.Settings.flow_log_retention_days</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Flow logs on, 90-day retention.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3445,14 +3781,10 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>05_Network.CloudFirewall; 09_CFW.Settings.enable_attack_alarm; 09_CFW.Settings.enable_traffic_alarm; 09_CFW.Settings.alarm_topic_name; 09_CFW.Settings.enable_anti_virus</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>IPS observe mode, alarms on to the ops topic, pay-per-use.</t>
-        </is>
-      </c>
+          <t>09_CFW.Settings</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3472,12 +3804,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>07_Security.Settings; 07_Security.SecMasterModules; 07_Security.AlertRules</t>
+          <t>05_Network.CloudFirewall; 09_CFW.Settings.enable_attack_alarm; 09_CFW.Settings.enable_traffic_alarm; 09_CFW.Settings.alarm_topic_name; 09_CFW.Settings.enable_anti_virus</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SecMaster in the security account; HSS/DBSS deferred.</t>
+          <t>IPS observe mode, alarms on to the ops topic, pay-per-use.</t>
         </is>
       </c>
     </row>
@@ -3499,24 +3831,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>04_Perimeter.SCPs</t>
+          <t>07_Security.Settings; 07_Security.SecMasterModules; 07_Security.AlertRules</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>The 8 LZ baseline guardrails, staged (created, not enforced).</t>
+          <t>SecMaster in the security account; HSS/DBSS deferred.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>C24</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3526,19 +3858,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>07_Security.WAF; 07_Security.WAFDomains</t>
+          <t>04_Perimeter.SCPs</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WAF off until an internet-facing app needs it.</t>
+          <t>The 8 LZ baseline guardrails, staged (created, not enforced).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3553,19 +3885,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>07_Security.AntiDDoS</t>
+          <t>07_Security.WAF; 07_Security.WAFDomains</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Default Anti-DDoS thresholds, no per-EIP tuning.</t>
+          <t>WAF off until an internet-facing app needs it.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3580,19 +3912,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>09_CFW.BlackWhiteLists; 09_CFW.DomainGroups</t>
+          <t>07_Security.AntiDDoS</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>No seed lists; firewall starts with the rule baseline only.</t>
+          <t>Default Anti-DDoS thresholds, no per-EIP tuning.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3607,19 +3939,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>06_Observability.AuditSettings.kms_audit_alias</t>
+          <t>09_CFW.BlackWhiteLists; 09_CFW.DomainGroups</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Platform-managed KMS keys per sensitive bucket.</t>
+          <t>No seed lists; firewall starts with the rule baseline only.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>D17</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3634,39 +3966,39 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>04_Perimeter.SCPs.ExceptionTagKey</t>
+          <t>06_Observability.AuditSettings.kms_audit_alias</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Public storage denied outright, no exception path.</t>
+          <t>Platform-managed KMS keys per sensitive bucket.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C24</t>
+          <t>D17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Compliance &amp; Audit</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>06_Observability.AuditSettings</t>
+          <t>04_Perimeter.SCPs.ExceptionTagKey</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Org-wide audit trail to the security account, 365-day retention.</t>
+          <t>Public storage denied outright, no exception path.</t>
         </is>
       </c>
     </row>
@@ -3688,12 +4020,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>04_Perimeter.ConfigConformancePacks</t>
+          <t>06_Observability.AuditSettings</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Landing Zone best-practice pack only.</t>
+          <t>Org-wide audit trail to the security account, 365-day retention.</t>
         </is>
       </c>
     </row>
@@ -3715,24 +4047,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>04_Perimeter.ConfigSetup</t>
+          <t>04_Perimeter.ConfigConformancePacks</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Config recorder + org aggregator in the security account.</t>
+          <t>Landing Zone best-practice pack only.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>C27</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3742,39 +4074,39 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>04_Perimeter.ConfigConformancePacks.ExcludedAccounts</t>
+          <t>04_Perimeter.ConfigSetup</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>No exemptions.</t>
+          <t>Config recorder + org aggregator in the security account.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>C27</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Operations &amp; Monitoring</t>
+          <t>Compliance &amp; Audit</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>06_Observability.OpsSettings; 06_Observability.OneClickNamespaces</t>
+          <t>04_Perimeter.ConfigConformancePacks.ExcludedAccounts</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Cloud Eye baseline bundles on core services, alerts to one ops topic.</t>
+          <t>No exemptions.</t>
         </is>
       </c>
     </row>
@@ -3796,12 +4128,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>06_Observability.LogAggregation</t>
+          <t>06_Observability.OpsSettings; 06_Observability.OneClickNamespaces</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>All platform logs converge centrally and archive to OBS.</t>
+          <t>Cloud Eye baseline bundles on core services, alerts to one ops topic.</t>
         </is>
       </c>
     </row>
@@ -3823,24 +4155,24 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>06_Observability.LogAggregation.archive_retention_days; 06_Observability.AuditSettings.audit_retention_days</t>
+          <t>06_Observability.LogAggregation</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>90-day hot, 365-day archive.</t>
+          <t>All platform logs converge centrally and archive to OBS.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>C30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3850,15 +4182,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>06_Observability.Subscribers; 06_Observability.OpsSettings.topic_name</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr"/>
+          <t>06_Observability.LogAggregation.archive_retention_days; 06_Observability.AuditSettings.audit_retention_days</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>90-day hot, 365-day archive.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3873,19 +4209,15 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>06_Observability.LogAggregation.enable_log_aggregation</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>No SIEM integration.</t>
-        </is>
-      </c>
+          <t>06_Observability.Subscribers; 06_Observability.OpsSettings.topic_name</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3898,37 +4230,37 @@
           <t>Operations &amp; Monitoring</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>06_Observability.LogAggregation.enable_log_aggregation</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Recorded for the workload phase; no platform default.</t>
+          <t>No SIEM integration.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>C30</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Finance &amp; Cost Management</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>02_Finance.Settings</t>
-        </is>
-      </c>
+          <t>Operations &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Central billing from the management account.</t>
+          <t>Recorded for the workload phase; no platform default.</t>
         </is>
       </c>
     </row>
@@ -3950,24 +4282,24 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>02_Finance.CostCenters</t>
+          <t>02_Finance.Settings</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Cost centres per business unit, prod/dev typed.</t>
+          <t>Central billing from the management account.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3982,19 +4314,19 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Platform costs absorbed centrally.</t>
+          <t>Cost centres per business unit, prod/dev typed.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>core</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4004,53 +4336,61 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>06_Observability.Subscribers</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
+          <t>02_Finance.CostCenters; 03_Identity.AppPermissionSets</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>One EP per application per environment tier, derived from the workload list; flagged for review.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>appendix</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Accounts &amp; Environments (optional)</t>
+          <t>Finance &amp; Cost Management</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>01_Foundation.WorkloadAccounts; 01_Foundation.OrganizationalUnits</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
+          <t>02_Finance.CostCenters</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Platform costs absorbed centrally.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>appendix</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>IP Plan (optional)</t>
+          <t>Finance &amp; Cost Management</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>05_Network.Settings.spoke_private_supernet; 05_Network.HubVPCs; 05_Network.HubSubnets; 05_Network.SpokeVPCs; 05_Network.SpokeSubnets</t>
+          <t>06_Observability.Subscribers</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -4058,7 +4398,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4068,12 +4408,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Teams &amp; Access (optional)</t>
+          <t>Accounts &amp; Environments (optional)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>03_Identity.Groups; 03_Identity.Users; 03_Identity.PermissionSets; 03_Identity.AccountAssignments</t>
+          <t>01_Foundation.WorkloadAccounts; 01_Foundation.OrganizationalUnits</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -4081,21 +4421,67 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>appendix</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>IP Plan (optional)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>05_Network.Settings.spoke_private_supernet; 05_Network.HubVPCs; 05_Network.HubSubnets; 05_Network.SpokeVPCs; 05_Network.SpokeSubnets</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>appendix</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Teams &amp; Access (optional)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>03_Identity.Groups; 03_Identity.Users; 03_Identity.PermissionSets; 03_Identity.AccountAssignments</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>_meta</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>meta</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr">
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
         <is>
           <t>questionnaire_version=1.0; schema_version=2.2</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
questionnaire: humanized wording pass (v1.1) from proofread review
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017p3Gy6G8WQ79VLPjM41ST5
</commit_message>
<xml_diff>
--- a/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
+++ b/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
@@ -537,14 +537,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="62" customHeight="1">
+          <t>Before you start</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>This questionnaire collects the information needed to design your Huawei Cloud Landing Zone: the governed multi-account foundation (organization, identity, network, security, audit and cost management) your workloads will land on. Your answers drive a draft design and configuration; anything unanswered becomes an explicit decision list we walk through together.</t>
+          <t>This questionnaire helps us understand how you want Huawei Cloud to be organized, secured, connected, and operated. You do not need to have every answer today. We use your responses to prepare a first design, then review assumptions and open decisions with you.</t>
         </is>
       </c>
     </row>
@@ -554,35 +554,35 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>How to answer</t>
+          <t>How to complete it</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>- Answer in free text, in as much or as little detail as you have. Attach diagrams, inventories or policies wherever they exist - a document beats retyping.</t>
+          <t>- Write as much or as little as you know. If you already have diagrams, inventories, standards, or policies, attach them instead of retyping the same information.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>- 'Unknown' and 'no requirement' are valid answers. Please answer every question on the Core Questions sheet; answer Deep-Dive questions only where they apply to you.</t>
+          <t>- “Unknown”, “not decided yet”, and “no specific requirement” are all valid answers. Please complete the Core Questions and use the Deep-Dive Questions only where they apply.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>- Anything left blank on the Deep-Dive sheet is designed to a documented Huawei best-practice default, which you review before anything is built.</t>
+          <t>- If a Deep-Dive question does not apply or is left blank, we will propose a sensible starting point and confirm it with you before implementation.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>- Appendices A-C are optional tables for facts that fit rows better than prose (accounts, IP ranges, teams). Fill what you know.</t>
+          <t>- Appendices A to C are optional. Use them when accounts, IP ranges, or team access are easier to describe in a table.</t>
         </is>
       </c>
     </row>
@@ -592,35 +592,35 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>What happens next</t>
+          <t>What happens after this</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>1. We convert your answers into a draft Landing Zone configuration.</t>
+          <t>1. We review your answers and prepare a draft landing zone design.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2. Open points and defaults come back to you as a short decision list.</t>
+          <t>2. We highlight anything that is unclear, undecided, or needs your approval.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3. A workshop resolves the decision list and finalizes the design (LLD).</t>
+          <t>3. We review those items with you and finalize the detailed design.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>4. The landing zone is built from that configuration - no console clicking.</t>
+          <t>4. The agreed design becomes the baseline for implementation and automation.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Version 1.0 - generated 2026-09-01 - schema 2.2</t>
+          <t>Version 1.1 - generated 2026-09-01 - schema 2.2</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Huawei Cloud Landing Zone Assessment - Core Questions - please answer all</t>
+          <t>Huawei Cloud Landing Zone Assessment - Core Questions</t>
         </is>
       </c>
     </row>
@@ -707,12 +707,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Describe your current cloud footprint: which providers you use (AWS, Azure, GCP, Alibaba, Huawei), roughly how many accounts / subscriptions / projects, and what each is for.</t>
+          <t>What does your cloud environment look like today? Please list the cloud providers you use, roughly how many accounts, subscriptions, or projects you have, and what they are used for.</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Free text; attach an account inventory or org chart if you have one. This shapes the account and OU structure we propose.</t>
+          <t>A simple summary is enough. If you already have an account inventory or organization diagram, attach it instead of retyping the details.</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>If you already have Huawei Cloud accounts, what runs in them today? Would you accept a fresh set of Landing Zone accounts, with existing workloads migrated or redeployed into them?</t>
+          <t>Do you already use Huawei Cloud? If yes, what is running there today, and are any existing accounts expected to remain in the future landing zone?</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Greenfield accounts give the cleanest governance baseline. If some accounts must be adopted as-is, list them and what they host.</t>
+          <t>We can design around existing accounts where needed. A new account structure is usually simpler to govern, but migration constraints may require a mixed approach.</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="E5" s="9" t="n"/>
     </row>
-    <row r="6" ht="76" customHeight="1">
+    <row r="6" ht="62" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>C3</t>
@@ -753,12 +753,12 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Which applications or workloads move to Huawei Cloud in the first wave? For each, which environments do you run (dev / test / UAT / production), and should each environment be isolated in its own account?</t>
+          <t>Which applications or workloads are in the first migration or deployment wave? For each one, tell us which environments you run, such as dev, test, UAT, and production.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Appendix A (Accounts &amp; Environments) has a table for this if you prefer rows over prose. Per-environment accounts are our recommended isolation boundary.</t>
+          <t>You can use Appendix A if a table is easier. Also tell us whether you prefer separate accounts for each environment or another isolation model.</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="E6" s="9" t="n"/>
     </row>
-    <row r="7" ht="76" customHeight="1">
+    <row r="7" ht="62" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>C4</t>
@@ -776,12 +776,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>If you built a landing zone or account hierarchy on another cloud (AWS OUs, Azure management groups, GCP folders), describe it. What worked well and what would you change?</t>
+          <t>Do you already have a landing zone or cloud account hierarchy elsewhere, such as Azure management groups or AWS Organizations? What would you like to keep or improve?</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>A diagram or export is ideal. We mirror proven structure where it fits Huawei Organizations.</t>
+          <t>A diagram or export is useful. We can reuse governance patterns that already work well for your teams.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Which Huawei Cloud region is your primary deployment region, and do you have secondary-region or disaster-recovery ambitions? Any data-residency constraints on where data may live?</t>
+          <t>Which Huawei Cloud region will be your primary region? Do you need a secondary region for disaster recovery, and are there any data residency requirements?</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>e.g. ap-southeast-3 (Singapore) primary. Residency constraints become an org-wide region guardrail.</t>
+          <t>For example, Singapore may be the primary region with another approved region reserved for DR. Residency requirements may also affect organization-wide controls.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Which teams will work in the cloud (platform, application, security, network, database, finance, ...) and what is each team responsible for?</t>
+          <t>Which teams will use or manage Huawei Cloud, and what is each team responsible for?</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Appendix C (Teams &amp; Access) has a table for this. Teams map to Identity Center groups and permission sets.</t>
+          <t>Typical teams include platform, application, security, network, database, finance, and audit. Appendix C can be used if you prefer a table.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="E12" s="9" t="n"/>
     </row>
-    <row r="13" ht="90" customHeight="1">
+    <row r="13" ht="62" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>C9</t>
@@ -898,12 +898,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>How should people sign in to Huawei Cloud: federated through your corporate identity provider (Entra ID / AD FS / Okta / other), or as natively managed Identity Center users? Which IdP product and version do you run?</t>
+          <t>How do you want users to sign in to Huawei Cloud? For example, through Microsoft Entra ID, AD FS, Okta, another identity provider, or Huawei Cloud-managed users.</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Federation keeps joiner-mover-leaver in your IdP. Native IC users need no IdP integration but are managed separately.</t>
+          <t>If you use an external identity provider, please include the product and version where known.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="E13" s="9" t="n"/>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="62" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>C10</t>
@@ -921,12 +921,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Does your identity provider support SAML 2.0 for sign-in and SCIM for automatic user/group provisioning?</t>
+          <t>If you plan to federate sign-in, does your identity provider support SAML 2.0 and SCIM provisioning?</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Both supported: full federation with auto-provisioning. SAML only: federation with manual user sync.</t>
+          <t>SAML provides federated sign-in. SCIM can automate user and group provisioning. If you are unsure, your identity team can confirm this later.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="E14" s="9" t="n"/>
     </row>
-    <row r="15" ht="76" customHeight="1">
+    <row r="15" ht="62" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>C11</t>
@@ -944,12 +944,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Do third parties (vendors, MSPs, auditors, outsourced developers) need access? Who, to which accounts or applications, at what permission level, and standing or time-boxed?</t>
+          <t>Will vendors, MSPs, auditors, or other third parties need access to Huawei Cloud? If yes, what should they access and for how long?</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Third-party access gets its own groups and least-privilege permission sets so it can be revoked cleanly.</t>
+          <t>Please include the expected permission level and whether access should be permanent or time-limited.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -967,12 +967,12 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>What password, MFA and session policies must the cloud enforce? (minimum length, expiry, MFA mandatory for whom, console session timeout, lockout rules)</t>
+          <t>What identity security policies must Huawei Cloud follow for passwords, MFA, account lockout, and session timeouts?</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>If you have no written policy, we apply the LZ baseline: 12+ character passwords, 90-day expiry, MFA required, 8-hour sessions, 60-minute console timeout.</t>
+          <t>If your organization already has an identity or access policy, attach it. If not, we can propose a baseline for review rather than asking you to define every setting now.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Describe your current network: data centres, offices, existing cloud networks, and how they interconnect. Attach a topology diagram if one exists.</t>
+          <t>Please describe your current network at a high level. Include data centres, offices, existing cloud networks, and how they connect today.</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Even a rough sketch helps. This anchors the hub-and-spoke design and interconnect plan.</t>
+          <t>A topology diagram is preferred if you have one. A rough diagram is also fine at this stage.</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="E18" s="9" t="n"/>
     </row>
-    <row r="19" ht="76" customHeight="1">
+    <row r="19" ht="62" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>C14</t>
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Which connectivity do you need between Huawei Cloud and your on-premises sites or other clouds? Private line (Direct Connect), site-to-site VPN, or both - and does the link need high availability?</t>
+          <t>How should Huawei Cloud connect to your data centres, offices, or other clouds? Do you expect Direct Connect, site-to-site VPN, or both?</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>List each site/cloud that must reach Huawei Cloud. VPN specifics (devices, IPs, routing) come in the deep-dive section.</t>
+          <t>For each connection, note whether high availability is required. Detailed VPN and routing information is covered in the deep-dive section.</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E19" s="9" t="n"/>
     </row>
-    <row r="20" ht="76" customHeight="1">
+    <row r="20" ht="62" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>C15</t>
@@ -1043,12 +1043,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>How should internet access work? Which applications need outbound internet, which must be reachable from the internet, and is centralized egress through a hub NAT + firewall acceptable?</t>
+          <t>How should internet connectivity work for your workloads? Which systems need outbound internet access, and which applications need to be reachable from the internet?</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Centralized egress is the LZ default: all spoke traffic exits through the inspected hub. Exceptions need a stated reason.</t>
+          <t>Also tell us whether you are comfortable centralizing internet egress through a shared NAT and firewall. We can review exceptions where needed.</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>The design connects VPCs hub-and-spoke through an Enterprise Router, which charges per attachment and per GB of traffic. Any objection, or constraints on inter-VPC bandwidth or cost?</t>
+          <t>Do you have any requirements or concerns for connectivity between VPCs, such as bandwidth, latency, traffic inspection, or cost?</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>The alternative (VPC peering mesh) does not scale with accounts and bypasses central inspection.</t>
+          <t>A common design uses Enterprise Router for hub-and-spoke connectivity and centralized inspection. We will confirm whether that pattern fits your traffic and cost requirements.</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E21" s="9" t="n"/>
     </row>
-    <row r="22" ht="90" customHeight="1">
+    <row r="22" ht="62" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>C17</t>
@@ -1089,12 +1089,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>IP addressing: can you allocate Huawei Cloud a dedicated private supernet (e.g. a /16 or larger) that overlaps nothing on-premises or in other clouds? Should your team or Huawei plan the per-VPC subnets within it?</t>
+          <t>Can you allocate a dedicated private IP range to Huawei Cloud that does not overlap with your existing networks? If yes, what range is available?</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Appendix B (IP Plan) has a table for known allocations and ranges to avoid. We recommend one supernet, centrally carved.</t>
+          <t>Appendix B can be used to list available and reserved ranges. We can either work from a customer-provided subnet plan or propose one for review.</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="E22" s="9" t="n"/>
     </row>
-    <row r="23" ht="62" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>C18</t>
@@ -1112,12 +1112,12 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>How many VPCs do you expect per account - one per account, one per environment, or several per application? Any reason to deviate from one VPC per workload account?</t>
+          <t>How do you expect VPCs to be organized across accounts and applications?</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>One VPC per workload account is the LZ default; the account boundary already isolates environments.</t>
+          <t>For example, you may use one VPC per workload account, multiple VPCs for separate applications, or another model. Tell us about any isolation requirements that influence this choice.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E23" s="9" t="n"/>
     </row>
-    <row r="24" ht="76" customHeight="1">
+    <row r="24" ht="62" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
         <is>
           <t>C19</t>
@@ -1135,12 +1135,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Which applications must communicate with each other, and which must be isolated? If you have a communication matrix (source, destination, port, protocol), attach it.</t>
+          <t>Which applications or environments need to communicate with each other, and which must stay isolated?</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>This drives firewall policy and security-group rules. No matrix: state the rule of thumb, e.g. 'prod isolated from non-prod; shared services reachable by all'.</t>
+          <t>If you have a source, destination, port, and protocol matrix, attach it. Otherwise, a few high-level rules are enough for the first design.</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="E24" s="9" t="n"/>
     </row>
-    <row r="25" ht="76" customHeight="1">
+    <row r="25" ht="48" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>C20</t>
@@ -1158,12 +1158,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Which tags must every cloud resource carry (e.g. project, owner, environment, cost-centre), and should resource creation be blocked when mandatory tags are missing?</t>
+          <t>Which tags should be mandatory on cloud resources, such as application, owner, environment, project, or cost centre?</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Tag keys/values feed cost allocation and the tag-enforcement guardrail. Blocking untagged creation is strict but keeps the estate clean from day one.</t>
+          <t>Also tell us whether missing tags should block deployment or only generate a compliance finding.</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Which security products do you use today (perimeter firewalls, EDR, SIEM, vulnerability management, PAM), and which must carry over or integrate with the cloud?</t>
+          <t>Which security tools do you use today, and which of them need to integrate with Huawei Cloud?</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>e.g. an existing PAM/bastion that must reach cloud servers, or an IPS policy to replicate.</t>
+          <t>Examples include firewalls, endpoint security, SIEM, vulnerability management, privileged access management, and security monitoring platforms.</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E27" s="9" t="n"/>
     </row>
-    <row r="28" ht="104" customHeight="1">
+    <row r="28" ht="76" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>C22</t>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Cloud Firewall expectations: should intrusion prevention observe first or block immediately? Do you want antivirus scanning at the perimeter? Should the firewall notify on attack detections and high traffic - and to whom? Billing: pay-per-use or monthly subscription?</t>
+          <t>What are your expectations for Cloud Firewall? Please cover intrusion prevention, perimeter antivirus if required, alerting, and any preferred billing model.</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Default rollout: IPS in observe mode first, then block after tuning; attack + high-traffic alerts to the ops mailbox; pay-per-use until sizing is proven.</t>
+          <t>If you do not have a defined policy yet, we can propose an initial observe-and-tune approach before moving selected protections into blocking mode.</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="E28" s="9" t="n"/>
     </row>
-    <row r="29" ht="76" customHeight="1">
+    <row r="29" ht="62" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>C23</t>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Do you need a cloud security-operations workspace (SecMaster) for centralized alerts and incident handling? Host security (HSS) on servers? Database security (DBSS)? Who consumes the alerts day-to-day?</t>
+          <t>Which Huawei Cloud security services do you expect to use, if any, such as SecMaster, Host Security Service, or Database Security Service? Who will review the alerts?</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>SecMaster carries a monthly cost per workspace; HSS/DBSS are per-instance quotas.</t>
+          <t>It is fine to mark this as undecided. We can recommend services based on your workload and compliance requirements.</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="E29" s="9" t="n"/>
     </row>
-    <row r="30" ht="90" customHeight="1">
+    <row r="30" ht="62" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
           <t>C24</t>
@@ -1257,12 +1257,12 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Which actions should be hard-blocked organization-wide, for everyone including admins? Examples: leaving the organization, disabling audit logging, making storage public, creating resources outside approved regions.</t>
+          <t>Are there actions that should be blocked across the whole organization, even for administrators?</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>These become service control policies (guardrails). We stage them in dry-run first, then enforce.</t>
+          <t>Examples include disabling audit logging, making storage public, leaving the organization, or deploying resources in unapproved regions.</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -1287,12 +1287,12 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Must every action in every account be logged centrally, tamper-proof and searchable? How long must audit logs be retained (hot and archived)?</t>
+          <t>What are your audit logging requirements? Should activity from all accounts be centralized, protected from changes, and searchable? How long must logs be retained?</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Common answer: 1 year online + long-term archive. Drives the central audit trail, its bucket and retention tiers.</t>
+          <t>Please separate online or searchable retention from long-term archive retention if your policy defines both.</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Which regulatory or industry frameworks apply to you (e.g. MAS TRM, PDPA, PCI-DSS, ISO 27001, SOC 2), and do auditors need evidence reports from the cloud platform?</t>
+          <t>Which regulatory, security, or industry standards apply to this environment?</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Frameworks map to continuous-compliance rule packs evaluated against all accounts.</t>
+          <t>Examples include MAS TRM, PDPA, PCI DSS, ISO 27001, and SOC 2. Also tell us whether auditors need platform-generated evidence or reports.</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1333,12 +1333,12 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Do you run continuous compliance monitoring today (AWS Config rules, Azure Policy)? Which account/team should own compliance tooling and its findings on Huawei Cloud?</t>
+          <t>Do you use continuous compliance controls today, such as Azure Policy or AWS Config? Which team should own compliance monitoring and findings in Huawei Cloud?</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Typically the security account owns the recorder, aggregator and rule packs.</t>
+          <t>If you already have a security governance process, describe how cloud findings should feed into it.</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="76" customHeight="1">
+    <row r="36" ht="62" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
           <t>C28</t>
@@ -1363,12 +1363,12 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>How do you monitor infrastructure today: which metrics and logs are collected, with which tools (Zabbix, Prometheus, vendor consoles), and what alarm rules and on-call flow exist?</t>
+          <t>How do you monitor infrastructure today? Which monitoring tools, metrics, logs, alert rules, and on-call processes should carry over to Huawei Cloud?</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>We map existing practice onto Cloud Eye one-click monitoring bundles + an alerting topic.</t>
+          <t>We will use this to map existing operational practices to Huawei Cloud monitoring and alerting services.</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="E36" s="9" t="n"/>
     </row>
-    <row r="37" ht="62" customHeight="1">
+    <row r="37" ht="48" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
         <is>
           <t>C29</t>
@@ -1386,12 +1386,12 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Should logs and monitoring from all accounts aggregate into one central operations account? Which log types matter most (audit, firewall, DNS, flow, application)?</t>
+          <t>Do you want logs and monitoring data from multiple accounts collected centrally? If yes, which log types are most important?</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Central aggregation is the LZ default: member-account logs converge to the ops account and archive to object storage.</t>
+          <t>Common examples include audit, firewall, DNS, VPC flow, operating system, and application logs.</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Log retention: how long must each class of log stay hot/searchable, and how long in cheap archive storage? Any class that must move to deep archive after a period?</t>
+          <t>How long should each type of log remain searchable, archived, or moved to lower-cost storage?</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>e.g. searchable 90 days, archived 1 year, deep-archived beyond. Drives retention tiers per log class.</t>
+          <t>If different log classes have different retention periods, list them separately. Approximate targets are fine for the first design.</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -1431,7 +1431,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="62" customHeight="1">
+    <row r="40" ht="48" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
           <t>C31</t>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Who manages cloud spend? Is there a financial administrator, and are budgets issued and controlled from the management account?</t>
+          <t>Who owns cloud cost management and billing? Who needs visibility into budgets, forecasts, and account-level spend?</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Shapes billing-account setup and who gets cost visibility.</t>
+          <t>Please include the finance or cloud governance teams that should receive budget notifications or reports.</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="E40" s="9" t="n"/>
     </row>
-    <row r="41" ht="62" customHeight="1">
+    <row r="41" ht="76" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
         <is>
           <t>C32</t>
@@ -1462,12 +1462,12 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Must cloud costs be allocated within your organization? Along which dimensions - business unit, department, project, environment, owner?</t>
+          <t>How should Huawei Cloud costs be allocated internally?</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Dimensions become cost-centre enterprise projects + the tag plan from the Network section.</t>
+          <t>Common dimensions include business unit, department, application, project, environment, and owner. We can align this with your tagging and account structure.</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -1534,7 +1534,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Huawei Cloud Landing Zone Assessment - Deep-Dive Questions - answer where applicable; blank = best-practice default</t>
+          <t>Huawei Cloud Landing Zone Assessment - Deep-Dive Questions - answer where relevant</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="62" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>D1</t>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>How do you expect the account estate to grow over the next 12-24 months - new workloads, business units, or countries? Who approves creating a new account?</t>
+          <t>How do you expect your Huawei Cloud account estate to grow over the next 12 to 24 months? Who should approve new accounts?</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Growth expectations size the OU structure and the account-vending process.</t>
+          <t>Consider new workloads, teams, business units, countries, acquisitions, or temporary project accounts.</t>
         </is>
       </c>
       <c r="D4" s="8" t="n"/>
@@ -1598,7 +1598,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
+    <row r="6" ht="76" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>D2</t>
@@ -1606,12 +1606,12 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Describe your CI/CD and automation landscape: which pipeline tools (GitHub Actions, GitLab, Jenkins, ...), where they run, and how automation should authenticate to Huawei Cloud (short-lived federated credentials vs long-lived access keys).</t>
+          <t>What CI/CD and automation tools do you use, and where do they run? How should pipelines authenticate to Huawei Cloud?</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>We strongly prefer OIDC/assume-role federation for pipelines; long-lived AK/SK is a last resort with rotation requirements.</t>
+          <t>Examples include GitHub Actions, GitLab, Jenkins, and Azure DevOps. Where possible, we prefer short-lived federated credentials over long-lived access keys.</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="E6" s="9" t="n"/>
     </row>
-    <row r="7" ht="62" customHeight="1">
+    <row r="7" ht="76" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>D3</t>
@@ -1629,12 +1629,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>How is emergency (break-glass) access handled today? Who holds root/master credentials, are they MFA-protected, and how is their use audited?</t>
+          <t>How do you handle emergency or break-glass access today?</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Informs custody of the management-account root user and the break-glass runbook.</t>
+          <t>Please describe who can use emergency credentials, how MFA is enforced, where credentials are stored, and how emergency access is reviewed or audited.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="E7" s="9" t="n"/>
     </row>
-    <row r="8" ht="90" customHeight="1">
+    <row r="8" ht="76" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>D4</t>
@@ -1652,12 +1652,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>How granular should permissions be? Are standard tiers (administrator / power user / read-only) per account enough, or do specific teams need permissions scoped to a single application's resources within a shared account?</t>
+          <t>How detailed do access permissions need to be? Are standard admin, power-user, and read-only roles enough, or do some teams need access limited to specific applications or resources?</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>App-scoped permission sets use enterprise-project scoping - more setup, tighter blast radius. Also note preferred session duration and a portal alias (the sign-in URL name) if you have one.</t>
+          <t>Also share any preferred session duration or sign-in portal naming requirements.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -1674,7 +1674,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
+    <row r="10" ht="62" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>D5</t>
@@ -1682,12 +1682,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>For each VPN site: what VPN device (vendor/model), does it have a static public IP, BGP or static routing (and your on-prem AS number), which on-prem subnets must be reachable, expected throughput, and do you want dual tunnels for HA?</t>
+          <t>For each site-to-site VPN, please provide the VPN device, public IP, routing method, on-premises networks, expected throughput, and availability requirements.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>One answer block per site is fine. BGP with dual tunnels is our recommended HA pattern.</t>
+          <t>If you use BGP, include your on-premises ASN. Dual tunnels with dynamic routing are usually preferred for high availability.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -1705,12 +1705,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>If you plan multiple regions: which traffic flows between them (replication, DR failover, user traffic) and with what bandwidth expectations?</t>
+          <t>If you plan to use more than one Huawei Cloud region, what traffic needs to move between regions and why?</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Skip if single-region.</t>
+          <t>Examples include data replication, DR failover, backup traffic, or user traffic. Include rough bandwidth needs where known.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="E11" s="9" t="n"/>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="62" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>D7</t>
@@ -1728,12 +1728,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Within each VPC, how should subnets be divided - by tier (web / app / db), by AZ, by size? Any sizing rules you follow today?</t>
+          <t>How should subnets be divided inside each VPC?</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Default: an app subnet and a db subnet per VPC, plus small platform subnets the design adds automatically.</t>
+          <t>Tell us whether you separate by application tier, availability zone, or another standard. Include any subnet sizing rules you already follow.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="E12" s="9" t="n"/>
     </row>
-    <row r="13" ht="76" customHeight="1">
+    <row r="13" ht="62" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>D8</t>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Do you run or plan Kubernetes/containers (CCE)? If yes: which workloads, and any preference on container networking? Container clusters consume IP space quickly - factor this into the IP plan.</t>
+          <t>Do you run or plan to run Kubernetes or containers on Huawei Cloud? If yes, which workloads are involved?</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Skip if no containers planned.</t>
+          <t>Container platforms can consume significant IP space, so early cluster estimates help us size the network correctly.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="E13" s="9" t="n"/>
     </row>
-    <row r="14" ht="104" customHeight="1">
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>D9</t>
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>DNS: which internal domains do you use, where are the authoritative servers, and must cloud workloads resolve on-prem names (or on-prem resolve cloud names)? Any public domains you want hosted on Huawei Cloud DNS?</t>
+          <t>How should DNS work between Huawei Cloud and your existing environment?</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>e.g. 'corp.internal on two on-prem DCs; cloud must resolve it; keep public zones at our registrar'. This shapes private zones, resolver endpoints and forwarding rules. Note whether DNS queries should be logged for security analytics.</t>
+          <t>Please include internal domain names, current DNS servers, required cloud-to-on-premises and on-premises-to-cloud resolution, public DNS hosting needs, and whether DNS query logging is required.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E14" s="9" t="n"/>
     </row>
-    <row r="15" ht="62" customHeight="1">
+    <row r="15" ht="76" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>D10</t>
@@ -1797,12 +1797,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>For internet-facing applications: which are published inbound, where should TLS terminate (load balancer / WAF / the app), and do you bring your own certificates?</t>
+          <t>Which applications will be exposed to the internet, and where should TLS terminate?</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Each published app becomes a load-balancer/DNAT entry behind the firewall, optionally fronted by WAF.</t>
+          <t>For each application, note whether TLS should terminate at the load balancer, WAF, or application, and whether you will provide existing certificates.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="E15" s="9" t="n"/>
     </row>
-    <row r="16" ht="62" customHeight="1">
+    <row r="16" ht="76" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>D11</t>
@@ -1820,12 +1820,12 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Expected internet bandwidth: rough outbound Mbit/s at peak, and how many public IPs you expect to need. Prefer paying by bandwidth (flat) or by traffic (per GB)?</t>
+          <t>What internet bandwidth and public IP capacity do you expect to need?</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Sizes the egress/ingress EIPs. Default: one 100 Mbit/s bandwidth-billed egress EIP, grown on demand.</t>
+          <t>A rough peak outbound bandwidth and estimated number of public IPs is enough. If you have a billing preference, note whether you prefer bandwidth-based or traffic-based charging.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -1843,12 +1843,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Do you need VPC flow logs (connection records for every VPC) for troubleshooting or security analytics, and how long should they be kept?</t>
+          <t>Do you need VPC flow logs for troubleshooting, security analysis, or compliance? If yes, how long should they be retained?</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Flow logs add LTS log volume/cost. Default: enabled, 90-day hot retention.</t>
+          <t>Flow logs increase log volume and storage cost, so retention should match the operational or compliance need.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -1873,12 +1873,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Web Application Firewall: which domains/applications need WAF protection, expected bandwidth and requests-per-second, and how are TLS certificates managed today?</t>
+          <t>Which internet-facing applications need Web Application Firewall protection?</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Skip if no internet-facing web apps. A dedicated WAF instance lives in the hub DMZ in front of the ingress load balancer.</t>
+          <t>For each application, provide the domain, rough bandwidth or request rate if known, and how TLS certificates are managed.</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -1896,12 +1896,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>DDoS: do any public endpoints need tuned traffic-cleaning thresholds or alerting when mitigation kicks in? Any history of DDoS incidents?</t>
+          <t>Do any public endpoints need specific DDoS thresholds, alerting, or enhanced protection?</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Basic Anti-DDoS is free per public IP; we tune thresholds and alarms per EIP.</t>
+          <t>If you have experienced DDoS incidents before, include the affected services and any traffic patterns you know.</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Do you maintain IP or domain block/allow lists (threat feeds, geo-blocking, known-bad IPs) that the cloud firewall should enforce from day one?</t>
+          <t>Do you maintain IP or domain allowlists, blocklists, threat feeds, or geo-blocking rules that should be carried into Huawei Cloud?</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Attach the lists or name the feed. These seed firewall blacklists/whitelists and domain groups.</t>
+          <t>Attach existing lists where possible. We can use them as input to firewall policy design.</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="E21" s="9" t="n"/>
     </row>
-    <row r="22" ht="62" customHeight="1">
+    <row r="22" ht="76" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>D16</t>
@@ -1942,12 +1942,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Encryption and key management: any requirements on who controls encryption keys (customer-managed KMS, BYOK), key rotation, or HSM-backed keys?</t>
+          <t>Do you have specific encryption or key-management requirements?</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>The LZ encrypts audit/log storage with dedicated KMS keys by default; BYOK changes key custody.</t>
+          <t>Examples include customer-managed KMS keys, BYOK, HSM-backed keys, key rotation periods, separation of key administrators, and audit requirements.</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -1965,12 +1965,12 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Is a public storage bucket ever legitimate for you (static websites, public downloads)? If yes, how should exceptions be approved and marked?</t>
+          <t>Will any object storage need to be publicly accessible?</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Default guardrail denies public storage outright; a tag-based exception path can be added with an approval process.</t>
+          <t>If yes, describe the use case and how exceptions should be approved. Otherwise, we can treat public storage as prohibited by default.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
+    <row r="25" ht="62" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>D18</t>
@@ -1995,12 +1995,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Should any accounts be exempt from compliance rule packs (sandboxes, short-lived POC accounts)? What makes an account exempt?</t>
+          <t>Should any accounts or environments be excluded from standard compliance checks?</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Exemptions reduce noise but create blind spots; name them explicitly.</t>
+          <t>Examples might include temporary sandboxes or proof-of-concept accounts. Please explain the reason and approval process for any exemption.</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="76" customHeight="1">
+    <row r="27" ht="62" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>D19</t>
@@ -2025,12 +2025,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Who should receive platform alerts, and how? List email addresses (or SMS numbers) per team/severity. Note: email subscribers must click a confirmation link before alerts flow.</t>
+          <t>Who should receive platform and security alerts, and through which channels?</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>These become subscriptions on the central alerting topic (also used by firewall and DDoS alarms).</t>
+          <t>List the relevant teams, email addresses, or other notification endpoints. You can also indicate different recipients by severity.</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -2048,12 +2048,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Do you integrate with a SIEM (Splunk, Sentinel, QRadar)? Which logs must reach it and by which ingestion method?</t>
+          <t>Do you use a SIEM such as Microsoft Sentinel, Splunk, or QRadar? Which Huawei Cloud logs should be sent to it?</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Cloud logs can be pulled from the central archive or streamed; the method affects the aggregation design.</t>
+          <t>If known, include your preferred ingestion method. We can confirm the technical integration during design.</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="E28" s="9" t="n"/>
     </row>
-    <row r="29" ht="76" customHeight="1">
+    <row r="29" ht="62" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>D21</t>
@@ -2071,12 +2071,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Backup and disaster recovery: what must be backed up (servers, databases, file/object data), with what RPO/RTO and retention? Any long-term archive requirement (e.g. move year-old backups to deep archive)?</t>
+          <t>What are your backup and disaster recovery requirements?</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>The LZ provisions the platform; workload backup policy is designed against these answers and lands with the workload rollout.</t>
+          <t>For each important workload, include what must be protected, target RPO and RTO, retention, and any long-term archive requirements.</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -2101,12 +2101,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>How should shared costs be handled - platform accounts (network hub, security, logging) and shared resources used by many departments? Showback, chargeback, or absorbed centrally?</t>
+          <t>How should shared cloud costs be handled?</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Common pattern: platform costs absorbed centrally or split pro-rata by consumption.</t>
+          <t>For shared network, security, logging, and platform services, tell us whether costs should be absorbed centrally, shown back to teams, or charged back.</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Do you have an existing Huawei Cloud commercial arrangement (enterprise agreement, partner/reseller, committed spend), and do you want budget alerts at defined thresholds sent to finance?</t>
+          <t>Do you have an existing Huawei Cloud commercial or billing arrangement?</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Commercial structure can constrain how accounts attach to billing; budget alerts reuse the ops alerting topic.</t>
+          <t>Examples include an enterprise agreement, partner or reseller arrangement, or committed spend. Also include any budget thresholds that should trigger finance alerts.</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>prod</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Account</t>
+          <t>Account / Environment</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -2478,7 +2478,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>(example) supernet</t>
+          <t>(example) Available supernet</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>Administrator</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>all accounts</t>
+          <t>All accounts</t>
         </is>
       </c>
       <c r="F4" s="10" t="n"/>
@@ -4478,7 +4478,7 @@
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>questionnaire_version=1.0; schema_version=2.2</t>
+          <t>questionnaire_version=1.1; schema_version=2.2</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: apply proofread wording to schema field help + doc generators
Ports the proofreading pass across the LLD schema notes/field help and the
config-book, IPAM, checklist and questionnaire generators; regenerates the
JSON schema and example questionnaire. Wording only, no behavior change.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017p3Gy6G8WQ79VLPjM41ST5
</commit_message>
<xml_diff>
--- a/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
+++ b/examples/HuaweiCloud-LZ-Assessment-Questionnaire.xlsx
@@ -822,12 +822,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>What email convention should account mailboxes follow? Each Huawei account needs a globally unique email address - do you have a pattern (e.g. cloud-&lt;account&gt;@yourco.com)?</t>
+          <t>What email address pattern should Huawei Cloud account mailboxes use? Each account needs a globally unique email address, for example cloud-&lt;account&gt;@yourco.com.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Plus-addressing (team+lz-prod@yourco.com) works if your mail system supports it.</t>
+          <t>Plus-addressing, such as team+lz-prod@yourco.com, works if your mail system supports it. If you do not have a pattern yet, we can propose one for review.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="E9" s="9" t="n"/>
     </row>
-    <row r="10" ht="104" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>C7</t>
@@ -845,12 +845,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Do you have a cloud resource naming convention (VPCs, subnets, gateways, buckets, vaults, log groups, ...)? State the pattern and an example, e.g. &lt;org&gt;-&lt;region&gt;-&lt;env&gt;-&lt;service&gt;-&lt;nn&gt; -&gt; acme-sg-prd-vpc-01.</t>
+          <t>Do you have a naming convention for cloud resources such as VPCs, subnets, gateways, buckets, and log groups? If yes, please share the pattern and an example, such as &lt;org&gt;-&lt;region&gt;-&lt;env&gt;-&lt;service&gt;-&lt;nn&gt; for acme-sg-prd-vpc-01.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Every named resource in the draft design is generated from this pattern, so one answer names the whole estate consistently. Note any hard limits (bucket names are globally unique and lowercase; some services cap length).</t>
+          <t>One answer lets us name every resource in the draft design consistently. Please note any hard limits, such as bucket names being globally unique and lowercase.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="E41" s="9" t="n"/>
     </row>
-    <row r="42" ht="104" customHeight="1">
+    <row r="42" ht="90" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
           <t>C33</t>
@@ -1485,12 +1485,12 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>How should resources be grouped INSIDE accounts using Enterprise Projects - Huawei's in-account grouping construct (closest analogue: Azure resource groups, or AWS tag-based resource groups)? By application, environment, department, cost centre - or do you have no preference?</t>
+          <t>How should resources be grouped inside accounts using Enterprise Projects, Huawei Cloud's in-account grouping construct? For example by application, environment, department, or cost centre. Enterprise Projects are similar to Azure resource groups.</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Enterprise projects scope both cost reporting and permissions (an admin can be limited to one EP), so the grouping outlives billing. No preference: the design derives an EP layout from your workload and cost-allocation answers.</t>
+          <t>Enterprise Projects scope both cost reporting and permissions, so the grouping outlives billing. If you have no preference, we derive a layout from your workload and cost-allocation answers.</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">

</xml_diff>